<commit_message>
Electricity sector input data updates
</commit_message>
<xml_diff>
--- a/InputData/elec/BCRbQ/BAU Cap Retirements before Quantization.xlsx
+++ b/InputData/elec/BCRbQ/BAU Cap Retirements before Quantization.xlsx
@@ -7072,13 +7072,13 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBECB8B3-0EEE-4E1E-9286-5C655BCF13DB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86CED531-7C58-42B2-A697-65582446CCA0}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEBEB933-E656-4020-859D-FF3117C80AF6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21D174A3-8339-452C-8CFB-781C70106DA0}"/>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8F813E1-0600-42BF-A463-280BEA76DF9D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7760B76-7A71-4615-B9D6-74FEA88FA45A}"/>
 </file>
</xml_diff>